<commit_message>
Release staff capabilities and negotiated pricing
</commit_message>
<xml_diff>
--- a/public/templates/orbit-staff-import.xlsx
+++ b/public/templates/orbit-staff-import.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importación Staff" sheetId="1" r:id="R1e067297158245b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R5901b5f127874e0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importación Staff" sheetId="1" r:id="R8c78481fb2d54203"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R8015ed616b72439a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -89,7 +89,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -116,8 +116,13 @@
         <x:fgColor rgb="FFFEF3C7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF59E0B"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="7">
+  <x:borders count="8">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -167,11 +172,25 @@
         <x:color rgb="FFE5E7EB"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD97706"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD97706"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD97706"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD97706"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="52">
+  <x:cellXfs count="56">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -279,6 +298,12 @@
     <x:xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -491,10 +516,11 @@
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="32" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="28" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -560,15 +586,18 @@
         <x:v>Capabilities</x:v>
       </x:c>
       <x:c r="J4" s="16" t="str">
+        <x:v>Specializations</x:v>
+      </x:c>
+      <x:c r="K4" s="16" t="str">
         <x:v>Notes</x:v>
       </x:c>
-      <x:c r="K4" s="16" t="str">
+      <x:c r="L4" s="16" t="str">
         <x:v>Bank</x:v>
       </x:c>
-      <x:c r="L4" s="16" t="str">
+      <x:c r="M4" s="17" t="str">
         <x:v>Account Number</x:v>
       </x:c>
-      <x:c r="M4" s="17" t="str">
+      <x:c r="N4" s="55" t="str">
         <x:v>Emergency Contact</x:v>
       </x:c>
     </x:row>
@@ -586,6 +615,7 @@
       <x:c r="K5" s="22"/>
       <x:c r="L5" s="25"/>
       <x:c r="M5" s="25"/>
+      <x:c r="N5"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="26"/>
@@ -601,6 +631,7 @@
       <x:c r="K6" s="23"/>
       <x:c r="L6" s="26"/>
       <x:c r="M6" s="26"/>
+      <x:c r="N6"/>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
       <x:c r="A7" s="26"/>
@@ -616,6 +647,7 @@
       <x:c r="K7" s="23"/>
       <x:c r="L7" s="26"/>
       <x:c r="M7" s="26"/>
+      <x:c r="N7"/>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="26"/>
@@ -631,6 +663,7 @@
       <x:c r="K8" s="23"/>
       <x:c r="L8" s="26"/>
       <x:c r="M8" s="26"/>
+      <x:c r="N8"/>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
       <x:c r="A9" s="26"/>
@@ -646,6 +679,7 @@
       <x:c r="K9" s="23"/>
       <x:c r="L9" s="26"/>
       <x:c r="M9" s="26"/>
+      <x:c r="N9"/>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="26"/>
@@ -661,6 +695,7 @@
       <x:c r="K10" s="23"/>
       <x:c r="L10" s="26"/>
       <x:c r="M10" s="26"/>
+      <x:c r="N10"/>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="26"/>
@@ -676,6 +711,7 @@
       <x:c r="K11" s="23"/>
       <x:c r="L11" s="26"/>
       <x:c r="M11" s="26"/>
+      <x:c r="N11"/>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="26"/>
@@ -691,6 +727,7 @@
       <x:c r="K12" s="23"/>
       <x:c r="L12" s="26"/>
       <x:c r="M12" s="26"/>
+      <x:c r="N12"/>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="26"/>
@@ -706,6 +743,7 @@
       <x:c r="K13" s="23"/>
       <x:c r="L13" s="26"/>
       <x:c r="M13" s="26"/>
+      <x:c r="N13"/>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="26"/>
@@ -721,6 +759,7 @@
       <x:c r="K14" s="23"/>
       <x:c r="L14" s="26"/>
       <x:c r="M14" s="26"/>
+      <x:c r="N14"/>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="26"/>
@@ -736,6 +775,7 @@
       <x:c r="K15" s="23"/>
       <x:c r="L15" s="26"/>
       <x:c r="M15" s="26"/>
+      <x:c r="N15"/>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="26"/>
@@ -751,6 +791,7 @@
       <x:c r="K16" s="23"/>
       <x:c r="L16" s="26"/>
       <x:c r="M16" s="26"/>
+      <x:c r="N16"/>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="26"/>
@@ -766,6 +807,7 @@
       <x:c r="K17" s="23"/>
       <x:c r="L17" s="26"/>
       <x:c r="M17" s="26"/>
+      <x:c r="N17"/>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="26"/>
@@ -781,6 +823,7 @@
       <x:c r="K18" s="23"/>
       <x:c r="L18" s="26"/>
       <x:c r="M18" s="26"/>
+      <x:c r="N18"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="26"/>
@@ -796,6 +839,7 @@
       <x:c r="K19" s="23"/>
       <x:c r="L19" s="26"/>
       <x:c r="M19" s="26"/>
+      <x:c r="N19"/>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="26"/>
@@ -811,6 +855,7 @@
       <x:c r="K20" s="23"/>
       <x:c r="L20" s="26"/>
       <x:c r="M20" s="26"/>
+      <x:c r="N20"/>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="26"/>
@@ -826,6 +871,7 @@
       <x:c r="K21" s="23"/>
       <x:c r="L21" s="26"/>
       <x:c r="M21" s="26"/>
+      <x:c r="N21"/>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
       <x:c r="A22" s="26"/>
@@ -841,6 +887,7 @@
       <x:c r="K22" s="23"/>
       <x:c r="L22" s="26"/>
       <x:c r="M22" s="26"/>
+      <x:c r="N22"/>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="A23" s="26"/>
@@ -856,6 +903,7 @@
       <x:c r="K23" s="23"/>
       <x:c r="L23" s="26"/>
       <x:c r="M23" s="26"/>
+      <x:c r="N23"/>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
       <x:c r="A24" s="26"/>
@@ -871,6 +919,7 @@
       <x:c r="K24" s="23"/>
       <x:c r="L24" s="26"/>
       <x:c r="M24" s="26"/>
+      <x:c r="N24"/>
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
       <x:c r="A25" s="26"/>
@@ -886,6 +935,7 @@
       <x:c r="K25" s="23"/>
       <x:c r="L25" s="26"/>
       <x:c r="M25" s="26"/>
+      <x:c r="N25"/>
     </x:row>
     <x:row r="26" ht="22" customHeight="1">
       <x:c r="A26" s="26"/>
@@ -901,6 +951,7 @@
       <x:c r="K26" s="23"/>
       <x:c r="L26" s="26"/>
       <x:c r="M26" s="26"/>
+      <x:c r="N26"/>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
       <x:c r="A27" s="26"/>
@@ -916,6 +967,7 @@
       <x:c r="K27" s="23"/>
       <x:c r="L27" s="26"/>
       <x:c r="M27" s="26"/>
+      <x:c r="N27"/>
     </x:row>
     <x:row r="28" ht="22" customHeight="1">
       <x:c r="A28" s="26"/>
@@ -931,6 +983,7 @@
       <x:c r="K28" s="23"/>
       <x:c r="L28" s="26"/>
       <x:c r="M28" s="26"/>
+      <x:c r="N28"/>
     </x:row>
     <x:row r="29" ht="22" customHeight="1">
       <x:c r="A29" s="26"/>
@@ -946,6 +999,7 @@
       <x:c r="K29" s="23"/>
       <x:c r="L29" s="26"/>
       <x:c r="M29" s="26"/>
+      <x:c r="N29"/>
     </x:row>
     <x:row r="30" ht="22" customHeight="1">
       <x:c r="A30" s="26"/>
@@ -961,6 +1015,7 @@
       <x:c r="K30" s="23"/>
       <x:c r="L30" s="26"/>
       <x:c r="M30" s="26"/>
+      <x:c r="N30"/>
     </x:row>
     <x:row r="31" ht="22" customHeight="1">
       <x:c r="A31" s="26"/>
@@ -976,6 +1031,7 @@
       <x:c r="K31" s="23"/>
       <x:c r="L31" s="26"/>
       <x:c r="M31" s="26"/>
+      <x:c r="N31"/>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
       <x:c r="A32" s="26"/>
@@ -991,6 +1047,7 @@
       <x:c r="K32" s="23"/>
       <x:c r="L32" s="26"/>
       <x:c r="M32" s="26"/>
+      <x:c r="N32"/>
     </x:row>
     <x:row r="33" ht="22" customHeight="1">
       <x:c r="A33" s="26"/>
@@ -1006,6 +1063,7 @@
       <x:c r="K33" s="23"/>
       <x:c r="L33" s="26"/>
       <x:c r="M33" s="26"/>
+      <x:c r="N33"/>
     </x:row>
     <x:row r="34" ht="22" customHeight="1">
       <x:c r="A34" s="26"/>
@@ -1021,6 +1079,7 @@
       <x:c r="K34" s="23"/>
       <x:c r="L34" s="26"/>
       <x:c r="M34" s="26"/>
+      <x:c r="N34"/>
     </x:row>
     <x:row r="35" ht="22" customHeight="1">
       <x:c r="A35" s="26"/>
@@ -1036,6 +1095,7 @@
       <x:c r="K35" s="23"/>
       <x:c r="L35" s="26"/>
       <x:c r="M35" s="26"/>
+      <x:c r="N35"/>
     </x:row>
     <x:row r="36" ht="22" customHeight="1">
       <x:c r="A36" s="26"/>
@@ -1051,6 +1111,7 @@
       <x:c r="K36" s="23"/>
       <x:c r="L36" s="26"/>
       <x:c r="M36" s="26"/>
+      <x:c r="N36"/>
     </x:row>
     <x:row r="37" ht="22" customHeight="1">
       <x:c r="A37" s="26"/>
@@ -1066,6 +1127,7 @@
       <x:c r="K37" s="23"/>
       <x:c r="L37" s="26"/>
       <x:c r="M37" s="26"/>
+      <x:c r="N37"/>
     </x:row>
     <x:row r="38" ht="22" customHeight="1">
       <x:c r="A38" s="26"/>
@@ -1081,6 +1143,7 @@
       <x:c r="K38" s="23"/>
       <x:c r="L38" s="26"/>
       <x:c r="M38" s="26"/>
+      <x:c r="N38"/>
     </x:row>
     <x:row r="39" ht="22" customHeight="1">
       <x:c r="A39" s="26"/>
@@ -1096,6 +1159,7 @@
       <x:c r="K39" s="23"/>
       <x:c r="L39" s="26"/>
       <x:c r="M39" s="26"/>
+      <x:c r="N39"/>
     </x:row>
     <x:row r="40" ht="22" customHeight="1">
       <x:c r="A40" s="26"/>
@@ -1111,6 +1175,7 @@
       <x:c r="K40" s="23"/>
       <x:c r="L40" s="26"/>
       <x:c r="M40" s="26"/>
+      <x:c r="N40"/>
     </x:row>
     <x:row r="41" ht="22" customHeight="1">
       <x:c r="A41" s="26"/>
@@ -1126,6 +1191,7 @@
       <x:c r="K41" s="23"/>
       <x:c r="L41" s="26"/>
       <x:c r="M41" s="26"/>
+      <x:c r="N41"/>
     </x:row>
     <x:row r="42" ht="22" customHeight="1">
       <x:c r="A42" s="26"/>
@@ -1141,6 +1207,7 @@
       <x:c r="K42" s="23"/>
       <x:c r="L42" s="26"/>
       <x:c r="M42" s="26"/>
+      <x:c r="N42"/>
     </x:row>
     <x:row r="43" ht="22" customHeight="1">
       <x:c r="A43" s="26"/>
@@ -1156,6 +1223,7 @@
       <x:c r="K43" s="23"/>
       <x:c r="L43" s="26"/>
       <x:c r="M43" s="26"/>
+      <x:c r="N43"/>
     </x:row>
     <x:row r="44" ht="22" customHeight="1">
       <x:c r="A44" s="26"/>
@@ -1171,6 +1239,7 @@
       <x:c r="K44" s="23"/>
       <x:c r="L44" s="26"/>
       <x:c r="M44" s="26"/>
+      <x:c r="N44"/>
     </x:row>
     <x:row r="45" ht="22" customHeight="1">
       <x:c r="A45" s="26"/>
@@ -1186,6 +1255,7 @@
       <x:c r="K45" s="23"/>
       <x:c r="L45" s="26"/>
       <x:c r="M45" s="26"/>
+      <x:c r="N45"/>
     </x:row>
     <x:row r="46" ht="22" customHeight="1">
       <x:c r="A46" s="26"/>
@@ -1201,6 +1271,7 @@
       <x:c r="K46" s="23"/>
       <x:c r="L46" s="26"/>
       <x:c r="M46" s="26"/>
+      <x:c r="N46"/>
     </x:row>
     <x:row r="47" ht="22" customHeight="1">
       <x:c r="A47" s="26"/>
@@ -1216,6 +1287,7 @@
       <x:c r="K47" s="23"/>
       <x:c r="L47" s="26"/>
       <x:c r="M47" s="26"/>
+      <x:c r="N47"/>
     </x:row>
     <x:row r="48" ht="22" customHeight="1">
       <x:c r="A48" s="26"/>
@@ -1231,6 +1303,7 @@
       <x:c r="K48" s="23"/>
       <x:c r="L48" s="26"/>
       <x:c r="M48" s="26"/>
+      <x:c r="N48"/>
     </x:row>
     <x:row r="49" ht="22" customHeight="1">
       <x:c r="A49" s="26"/>
@@ -1246,6 +1319,7 @@
       <x:c r="K49" s="23"/>
       <x:c r="L49" s="26"/>
       <x:c r="M49" s="26"/>
+      <x:c r="N49"/>
     </x:row>
     <x:row r="50" ht="22" customHeight="1">
       <x:c r="A50" s="26"/>
@@ -1261,6 +1335,7 @@
       <x:c r="K50" s="23"/>
       <x:c r="L50" s="26"/>
       <x:c r="M50" s="26"/>
+      <x:c r="N50"/>
     </x:row>
     <x:row r="51" ht="22" customHeight="1">
       <x:c r="A51" s="26"/>
@@ -1276,6 +1351,7 @@
       <x:c r="K51" s="23"/>
       <x:c r="L51" s="26"/>
       <x:c r="M51" s="26"/>
+      <x:c r="N51"/>
     </x:row>
     <x:row r="52" ht="22" customHeight="1">
       <x:c r="A52" s="26"/>
@@ -1291,6 +1367,7 @@
       <x:c r="K52" s="23"/>
       <x:c r="L52" s="26"/>
       <x:c r="M52" s="26"/>
+      <x:c r="N52"/>
     </x:row>
     <x:row r="53" ht="22" customHeight="1">
       <x:c r="A53" s="26"/>
@@ -1306,6 +1383,7 @@
       <x:c r="K53" s="23"/>
       <x:c r="L53" s="26"/>
       <x:c r="M53" s="26"/>
+      <x:c r="N53"/>
     </x:row>
     <x:row r="54" ht="22" customHeight="1">
       <x:c r="A54" s="26"/>
@@ -1321,6 +1399,7 @@
       <x:c r="K54" s="23"/>
       <x:c r="L54" s="26"/>
       <x:c r="M54" s="26"/>
+      <x:c r="N54"/>
     </x:row>
     <x:row r="55" ht="22" customHeight="1">
       <x:c r="A55" s="26"/>
@@ -1336,6 +1415,7 @@
       <x:c r="K55" s="23"/>
       <x:c r="L55" s="26"/>
       <x:c r="M55" s="26"/>
+      <x:c r="N55"/>
     </x:row>
     <x:row r="56" ht="22" customHeight="1">
       <x:c r="A56" s="26"/>
@@ -1351,6 +1431,7 @@
       <x:c r="K56" s="23"/>
       <x:c r="L56" s="26"/>
       <x:c r="M56" s="26"/>
+      <x:c r="N56"/>
     </x:row>
     <x:row r="57" ht="22" customHeight="1">
       <x:c r="A57" s="26"/>
@@ -1366,6 +1447,7 @@
       <x:c r="K57" s="23"/>
       <x:c r="L57" s="26"/>
       <x:c r="M57" s="26"/>
+      <x:c r="N57"/>
     </x:row>
     <x:row r="58" ht="22" customHeight="1">
       <x:c r="A58" s="26"/>
@@ -1381,6 +1463,7 @@
       <x:c r="K58" s="23"/>
       <x:c r="L58" s="26"/>
       <x:c r="M58" s="26"/>
+      <x:c r="N58"/>
     </x:row>
     <x:row r="59" ht="22" customHeight="1">
       <x:c r="A59" s="26"/>
@@ -1396,6 +1479,7 @@
       <x:c r="K59" s="23"/>
       <x:c r="L59" s="26"/>
       <x:c r="M59" s="26"/>
+      <x:c r="N59"/>
     </x:row>
     <x:row r="60" ht="22" customHeight="1">
       <x:c r="A60" s="26"/>
@@ -1411,6 +1495,7 @@
       <x:c r="K60" s="23"/>
       <x:c r="L60" s="26"/>
       <x:c r="M60" s="26"/>
+      <x:c r="N60"/>
     </x:row>
     <x:row r="61" ht="22" customHeight="1">
       <x:c r="A61" s="26"/>
@@ -1426,6 +1511,7 @@
       <x:c r="K61" s="23"/>
       <x:c r="L61" s="26"/>
       <x:c r="M61" s="26"/>
+      <x:c r="N61"/>
     </x:row>
     <x:row r="62" ht="22" customHeight="1">
       <x:c r="A62" s="26"/>
@@ -1441,6 +1527,7 @@
       <x:c r="K62" s="23"/>
       <x:c r="L62" s="26"/>
       <x:c r="M62" s="26"/>
+      <x:c r="N62"/>
     </x:row>
     <x:row r="63" ht="22" customHeight="1">
       <x:c r="A63" s="26"/>
@@ -1456,6 +1543,7 @@
       <x:c r="K63" s="23"/>
       <x:c r="L63" s="26"/>
       <x:c r="M63" s="26"/>
+      <x:c r="N63"/>
     </x:row>
     <x:row r="64" ht="22" customHeight="1">
       <x:c r="A64" s="26"/>
@@ -1471,6 +1559,7 @@
       <x:c r="K64" s="23"/>
       <x:c r="L64" s="26"/>
       <x:c r="M64" s="26"/>
+      <x:c r="N64"/>
     </x:row>
     <x:row r="65" ht="22" customHeight="1">
       <x:c r="A65" s="26"/>
@@ -1486,6 +1575,7 @@
       <x:c r="K65" s="23"/>
       <x:c r="L65" s="26"/>
       <x:c r="M65" s="26"/>
+      <x:c r="N65"/>
     </x:row>
     <x:row r="66" ht="22" customHeight="1">
       <x:c r="A66" s="26"/>
@@ -1501,6 +1591,7 @@
       <x:c r="K66" s="23"/>
       <x:c r="L66" s="26"/>
       <x:c r="M66" s="26"/>
+      <x:c r="N66"/>
     </x:row>
     <x:row r="67" ht="22" customHeight="1">
       <x:c r="A67" s="26"/>
@@ -1516,6 +1607,7 @@
       <x:c r="K67" s="23"/>
       <x:c r="L67" s="26"/>
       <x:c r="M67" s="26"/>
+      <x:c r="N67"/>
     </x:row>
     <x:row r="68" ht="22" customHeight="1">
       <x:c r="A68" s="26"/>
@@ -1531,6 +1623,7 @@
       <x:c r="K68" s="23"/>
       <x:c r="L68" s="26"/>
       <x:c r="M68" s="26"/>
+      <x:c r="N68"/>
     </x:row>
     <x:row r="69" ht="22" customHeight="1">
       <x:c r="A69" s="26"/>
@@ -1546,6 +1639,7 @@
       <x:c r="K69" s="23"/>
       <x:c r="L69" s="26"/>
       <x:c r="M69" s="26"/>
+      <x:c r="N69"/>
     </x:row>
     <x:row r="70" ht="22" customHeight="1">
       <x:c r="A70" s="26"/>
@@ -1561,6 +1655,7 @@
       <x:c r="K70" s="23"/>
       <x:c r="L70" s="26"/>
       <x:c r="M70" s="26"/>
+      <x:c r="N70"/>
     </x:row>
     <x:row r="71" ht="22" customHeight="1">
       <x:c r="A71" s="26"/>
@@ -1576,6 +1671,7 @@
       <x:c r="K71" s="23"/>
       <x:c r="L71" s="26"/>
       <x:c r="M71" s="26"/>
+      <x:c r="N71"/>
     </x:row>
     <x:row r="72" ht="22" customHeight="1">
       <x:c r="A72" s="26"/>
@@ -1591,6 +1687,7 @@
       <x:c r="K72" s="23"/>
       <x:c r="L72" s="26"/>
       <x:c r="M72" s="26"/>
+      <x:c r="N72"/>
     </x:row>
     <x:row r="73" ht="22" customHeight="1">
       <x:c r="A73" s="26"/>
@@ -1606,6 +1703,7 @@
       <x:c r="K73" s="23"/>
       <x:c r="L73" s="26"/>
       <x:c r="M73" s="26"/>
+      <x:c r="N73"/>
     </x:row>
     <x:row r="74" ht="22" customHeight="1">
       <x:c r="A74" s="26"/>
@@ -1621,6 +1719,7 @@
       <x:c r="K74" s="23"/>
       <x:c r="L74" s="26"/>
       <x:c r="M74" s="26"/>
+      <x:c r="N74"/>
     </x:row>
     <x:row r="75" ht="22" customHeight="1">
       <x:c r="A75" s="26"/>
@@ -1636,6 +1735,7 @@
       <x:c r="K75" s="23"/>
       <x:c r="L75" s="26"/>
       <x:c r="M75" s="26"/>
+      <x:c r="N75"/>
     </x:row>
     <x:row r="76" ht="22" customHeight="1">
       <x:c r="A76" s="26"/>
@@ -1651,6 +1751,7 @@
       <x:c r="K76" s="23"/>
       <x:c r="L76" s="26"/>
       <x:c r="M76" s="26"/>
+      <x:c r="N76"/>
     </x:row>
     <x:row r="77" ht="22" customHeight="1">
       <x:c r="A77" s="26"/>
@@ -1666,6 +1767,7 @@
       <x:c r="K77" s="23"/>
       <x:c r="L77" s="26"/>
       <x:c r="M77" s="26"/>
+      <x:c r="N77"/>
     </x:row>
     <x:row r="78" ht="22" customHeight="1">
       <x:c r="A78" s="26"/>
@@ -1681,6 +1783,7 @@
       <x:c r="K78" s="23"/>
       <x:c r="L78" s="26"/>
       <x:c r="M78" s="26"/>
+      <x:c r="N78"/>
     </x:row>
     <x:row r="79" ht="22" customHeight="1">
       <x:c r="A79" s="26"/>
@@ -1696,6 +1799,7 @@
       <x:c r="K79" s="23"/>
       <x:c r="L79" s="26"/>
       <x:c r="M79" s="26"/>
+      <x:c r="N79"/>
     </x:row>
     <x:row r="80" ht="22" customHeight="1">
       <x:c r="A80" s="26"/>
@@ -1711,6 +1815,7 @@
       <x:c r="K80" s="23"/>
       <x:c r="L80" s="26"/>
       <x:c r="M80" s="26"/>
+      <x:c r="N80"/>
     </x:row>
     <x:row r="81" ht="22" customHeight="1">
       <x:c r="A81" s="26"/>
@@ -1726,6 +1831,7 @@
       <x:c r="K81" s="23"/>
       <x:c r="L81" s="26"/>
       <x:c r="M81" s="26"/>
+      <x:c r="N81"/>
     </x:row>
     <x:row r="82" ht="22" customHeight="1">
       <x:c r="A82" s="26"/>
@@ -1741,6 +1847,7 @@
       <x:c r="K82" s="23"/>
       <x:c r="L82" s="26"/>
       <x:c r="M82" s="26"/>
+      <x:c r="N82"/>
     </x:row>
     <x:row r="83" ht="22" customHeight="1">
       <x:c r="A83" s="26"/>
@@ -1756,6 +1863,7 @@
       <x:c r="K83" s="23"/>
       <x:c r="L83" s="26"/>
       <x:c r="M83" s="26"/>
+      <x:c r="N83"/>
     </x:row>
     <x:row r="84" ht="22" customHeight="1">
       <x:c r="A84" s="26"/>
@@ -1771,6 +1879,7 @@
       <x:c r="K84" s="23"/>
       <x:c r="L84" s="26"/>
       <x:c r="M84" s="26"/>
+      <x:c r="N84"/>
     </x:row>
     <x:row r="85" ht="22" customHeight="1">
       <x:c r="A85" s="26"/>
@@ -1786,6 +1895,7 @@
       <x:c r="K85" s="23"/>
       <x:c r="L85" s="26"/>
       <x:c r="M85" s="26"/>
+      <x:c r="N85"/>
     </x:row>
     <x:row r="86" ht="22" customHeight="1">
       <x:c r="A86" s="26"/>
@@ -1801,6 +1911,7 @@
       <x:c r="K86" s="23"/>
       <x:c r="L86" s="26"/>
       <x:c r="M86" s="26"/>
+      <x:c r="N86"/>
     </x:row>
     <x:row r="87" ht="22" customHeight="1">
       <x:c r="A87" s="26"/>
@@ -1816,6 +1927,7 @@
       <x:c r="K87" s="23"/>
       <x:c r="L87" s="26"/>
       <x:c r="M87" s="26"/>
+      <x:c r="N87"/>
     </x:row>
     <x:row r="88" ht="22" customHeight="1">
       <x:c r="A88" s="26"/>
@@ -1831,6 +1943,7 @@
       <x:c r="K88" s="23"/>
       <x:c r="L88" s="26"/>
       <x:c r="M88" s="26"/>
+      <x:c r="N88"/>
     </x:row>
     <x:row r="89" ht="22" customHeight="1">
       <x:c r="A89" s="26"/>
@@ -1846,6 +1959,7 @@
       <x:c r="K89" s="23"/>
       <x:c r="L89" s="26"/>
       <x:c r="M89" s="26"/>
+      <x:c r="N89"/>
     </x:row>
     <x:row r="90" ht="22" customHeight="1">
       <x:c r="A90" s="26"/>
@@ -1861,6 +1975,7 @@
       <x:c r="K90" s="23"/>
       <x:c r="L90" s="26"/>
       <x:c r="M90" s="26"/>
+      <x:c r="N90"/>
     </x:row>
     <x:row r="91" ht="22" customHeight="1">
       <x:c r="A91" s="26"/>
@@ -1876,6 +1991,7 @@
       <x:c r="K91" s="23"/>
       <x:c r="L91" s="26"/>
       <x:c r="M91" s="26"/>
+      <x:c r="N91"/>
     </x:row>
     <x:row r="92" ht="22" customHeight="1">
       <x:c r="A92" s="26"/>
@@ -1891,6 +2007,7 @@
       <x:c r="K92" s="23"/>
       <x:c r="L92" s="26"/>
       <x:c r="M92" s="26"/>
+      <x:c r="N92"/>
     </x:row>
     <x:row r="93" ht="22" customHeight="1">
       <x:c r="A93" s="26"/>
@@ -1906,6 +2023,7 @@
       <x:c r="K93" s="23"/>
       <x:c r="L93" s="26"/>
       <x:c r="M93" s="26"/>
+      <x:c r="N93"/>
     </x:row>
     <x:row r="94" ht="22" customHeight="1">
       <x:c r="A94" s="26"/>
@@ -1921,6 +2039,7 @@
       <x:c r="K94" s="23"/>
       <x:c r="L94" s="26"/>
       <x:c r="M94" s="26"/>
+      <x:c r="N94"/>
     </x:row>
     <x:row r="95" ht="22" customHeight="1">
       <x:c r="A95" s="26"/>
@@ -1936,6 +2055,7 @@
       <x:c r="K95" s="23"/>
       <x:c r="L95" s="26"/>
       <x:c r="M95" s="26"/>
+      <x:c r="N95"/>
     </x:row>
     <x:row r="96" ht="22" customHeight="1">
       <x:c r="A96" s="26"/>
@@ -1951,6 +2071,7 @@
       <x:c r="K96" s="23"/>
       <x:c r="L96" s="26"/>
       <x:c r="M96" s="26"/>
+      <x:c r="N96"/>
     </x:row>
     <x:row r="97" ht="22" customHeight="1">
       <x:c r="A97" s="26"/>
@@ -1966,6 +2087,7 @@
       <x:c r="K97" s="23"/>
       <x:c r="L97" s="26"/>
       <x:c r="M97" s="26"/>
+      <x:c r="N97"/>
     </x:row>
     <x:row r="98" ht="22" customHeight="1">
       <x:c r="A98" s="26"/>
@@ -1981,6 +2103,7 @@
       <x:c r="K98" s="23"/>
       <x:c r="L98" s="26"/>
       <x:c r="M98" s="26"/>
+      <x:c r="N98"/>
     </x:row>
     <x:row r="99" ht="22" customHeight="1">
       <x:c r="A99" s="26"/>
@@ -1996,6 +2119,7 @@
       <x:c r="K99" s="23"/>
       <x:c r="L99" s="26"/>
       <x:c r="M99" s="26"/>
+      <x:c r="N99"/>
     </x:row>
     <x:row r="100" ht="22" customHeight="1">
       <x:c r="A100" s="26"/>
@@ -2011,6 +2135,7 @@
       <x:c r="K100" s="23"/>
       <x:c r="L100" s="26"/>
       <x:c r="M100" s="26"/>
+      <x:c r="N100"/>
     </x:row>
     <x:row r="101" ht="22" customHeight="1">
       <x:c r="A101" s="26"/>
@@ -2026,6 +2151,7 @@
       <x:c r="K101" s="23"/>
       <x:c r="L101" s="26"/>
       <x:c r="M101" s="26"/>
+      <x:c r="N101"/>
     </x:row>
     <x:row r="102" ht="22" customHeight="1">
       <x:c r="A102" s="26"/>
@@ -2041,6 +2167,7 @@
       <x:c r="K102" s="23"/>
       <x:c r="L102" s="26"/>
       <x:c r="M102" s="26"/>
+      <x:c r="N102"/>
     </x:row>
     <x:row r="103" ht="22" customHeight="1">
       <x:c r="A103" s="26"/>
@@ -2056,6 +2183,7 @@
       <x:c r="K103" s="23"/>
       <x:c r="L103" s="26"/>
       <x:c r="M103" s="26"/>
+      <x:c r="N103"/>
     </x:row>
     <x:row r="104" ht="22" customHeight="1">
       <x:c r="A104" s="27"/>
@@ -2071,6 +2199,7 @@
       <x:c r="K104" s="24"/>
       <x:c r="L104" s="27"/>
       <x:c r="M104" s="27"/>
+      <x:c r="N104"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2079,7 +2208,7 @@
   </x:mergeCells>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="G5:G104">
-      <x:formula1>'Instrucciones'!$B$10:$B$11</x:formula1>
+      <x:formula1>"ACTIVE,VACATION,MEDICAL_LEAVE,INACTIVE"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="H5:H104">
       <x:formula1>'Instrucciones'!$B$14:$B$15</x:formula1>

</xml_diff>